<commit_message>
Latest generated outputs 2026-08-10
</commit_message>
<xml_diff>
--- a/generated/spreadsheet/advertising-consent-advertising.xlsx
+++ b/generated/spreadsheet/advertising-consent-advertising.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I96"/>
+  <dimension ref="A1:I98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -435,9 +435,9 @@
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="72" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -1750,13 +1750,17 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
           <t>Address Text</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr"/>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>Text representation of an address or site</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -1785,13 +1789,17 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
           <t>Postcode</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>Postcode for a contact address or site</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -1815,14 +1823,22 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>UPRN</t>
+        </is>
+      </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>The name of a company (that the agent works for)</t>
+          <t>Unique Property Reference Number for a property</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -1846,19 +1862,19 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>User role</t>
+          <t>Company</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>The role of the named individual. Agent or proxy</t>
+          <t>The name of a company (that the agent works for)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -1868,58 +1884,58 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Applicant contact details</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Telephone number and email address of the applicant.</t>
-        </is>
-      </c>
+      <c r="A43" s="2" t="n"/>
+      <c r="B43" s="2" t="n"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Applicant reference</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr"/>
+          <t>agent</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>User role</t>
+        </is>
+      </c>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr"/>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Reference to match contact details to a named individual from the applicant details component</t>
+          <t>The role of the named individual. Agent or proxy</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
-      <c r="B44" s="2" t="n"/>
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Applicant contact details</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Telephone number and email address of the applicant.</t>
+        </is>
+      </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Contact details</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Email</t>
-        </is>
-      </c>
+          <t>Applicant reference</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>The email address that can be used for electronic correspondence with the individual</t>
+          <t>Reference to match contact details to a named individual from the applicant details component</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -1943,18 +1959,14 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Phone number(s)[]</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Phone number</t>
-        </is>
-      </c>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr"/>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -1964,7 +1976,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -1983,18 +1995,18 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Contact priority</t>
+          <t>Phone number</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>The priority of a number</t>
+          <t>A phone number</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2004,47 +2016,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>Applicant details</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Name and contact information for the parties making the application.</t>
-        </is>
-      </c>
+      <c r="A47" s="2" t="n"/>
+      <c r="B47" s="2" t="n"/>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Applicants[]</t>
+          <t>Contact details</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr"/>
+          <t>Phone number(s)[]</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Contact priority</t>
+        </is>
+      </c>
       <c r="F47" s="2" t="inlineStr"/>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>The priority of a number</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="B48" s="2" t="n"/>
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Applicant details</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Name and contact information for the parties making the application.</t>
+        </is>
+      </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Applicants[]</t>
@@ -2052,18 +2068,14 @@
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Person</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>The title of the individual</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -2073,7 +2085,7 @@
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2092,13 +2104,13 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>First Name</t>
+          <t>Title</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr"/>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>The first name of the individual</t>
+          <t>The title of the individual</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -2108,7 +2120,7 @@
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2127,13 +2139,13 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Last Name</t>
+          <t>First Name</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>The last name of the individual</t>
+          <t>The first name of the individual</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -2162,13 +2174,13 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Last Name</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr"/>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>The last name of the individual</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -2197,102 +2209,122 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Address Text</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Text representation of an address or site</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n"/>
+      <c r="B53" s="2" t="n"/>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Applicants[]</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
           <t>Postcode</t>
         </is>
       </c>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>The postal code</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>MAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>Postcode for a contact address or site</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n"/>
+      <c r="B54" s="2" t="n"/>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>Applicants[]</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Contact address</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>UPRN</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Unique Property Reference Number for a property</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>MAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Checklist</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Checking whether all the requirements of the form have been met, such as proof of payment or supporting documentation.</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>National requirement types[]</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>List of the document types required for the given application type</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Community consultation</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>What community consultation activities have taken place as part of the application</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>Have consulted</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Whether community consultation has been carried out</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>MUST</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n"/>
-      <c r="B55" s="2" t="n"/>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr"/>
@@ -2300,7 +2332,7 @@
       <c r="F55" s="2" t="inlineStr"/>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Provide details of the community consultation</t>
+          <t>List of the document types required for the given application type</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -2310,24 +2342,24 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Conflict of interest</t>
+          <t>Community consultation</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
+          <t>What community consultation activities have taken place as part of the application</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Conflict to declare</t>
+          <t>Have consulted</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr"/>
@@ -2335,7 +2367,7 @@
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Indicates whether any named applicant or agent has a relationship to the planning authority that must be declared</t>
+          <t>Whether community consultation has been carried out</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
@@ -2354,7 +2386,7 @@
       <c r="B57" s="2" t="n"/>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Person reference</t>
+          <t>Description</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr"/>
@@ -2362,7 +2394,7 @@
       <c r="F57" s="2" t="inlineStr"/>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Reference to the applicant or agent with the conflict</t>
+          <t>Provide details of the community consultation</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -2377,11 +2409,19 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
-      <c r="B58" s="2" t="n"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Conflict of interest</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Details of any conflict of interest that may exist between the applicant and planning authority.</t>
+        </is>
+      </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Conflict details</t>
+          <t>Conflict to declare</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr"/>
@@ -2389,34 +2429,26 @@
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Details of the conflict of interest including name, role and how the individual is related to the planning authority</t>
+          <t>Indicates whether any named applicant or agent has a relationship to the planning authority that must be declared</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Interest in land</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Whether the applicant owns or has permission to use the land where the proposed advertisement will be placed</t>
-        </is>
-      </c>
+      <c r="A59" s="2" t="n"/>
+      <c r="B59" s="2" t="n"/>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Applicant owns land</t>
+          <t>Person reference</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr"/>
@@ -2424,17 +2456,17 @@
       <c r="F59" s="2" t="inlineStr"/>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>True or False indicating whether the applicant owns the land where the advertisement will be displayed</t>
+          <t>Reference to the applicant or agent with the conflict</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I59" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2475,7 @@
       <c r="B60" s="2" t="n"/>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>Permission obtained</t>
+          <t>Conflict details</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr"/>
@@ -2451,12 +2483,12 @@
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>True or False indicating whether permission of the owner for the display of an advertisement has been obtained</t>
+          <t>Details of the conflict of interest including name, role and how the individual is related to the planning authority</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr">
@@ -2466,11 +2498,19 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
-      <c r="B61" s="2" t="n"/>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>Interest in land</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>Whether the applicant owns or has permission to use the land where the proposed advertisement will be placed</t>
+        </is>
+      </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Permission not obtained details</t>
+          <t>Applicant owns land</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr"/>
@@ -2478,34 +2518,26 @@
       <c r="F61" s="2" t="inlineStr"/>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Details explaining why permission from the land owner has not been obtained for the advertisement display</t>
+          <t>True or False indicating whether the applicant owns the land where the advertisement will be displayed</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Declaration</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Signed and dated verification of the application's accuracy.</t>
-        </is>
-      </c>
+      <c r="A62" s="2" t="n"/>
+      <c r="B62" s="2" t="n"/>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Person reference</t>
+          <t>Permission obtained</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr"/>
@@ -2513,17 +2545,17 @@
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Declaration must be made by an applicant or agent making the application</t>
+          <t>True or False indicating whether permission of the owner for the display of an advertisement has been obtained</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2564,7 @@
       <c r="B63" s="2" t="n"/>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>Declaration confirmed</t>
+          <t>Permission not obtained details</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr"/>
@@ -2540,26 +2572,34 @@
       <c r="F63" s="2" t="inlineStr"/>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
+          <t>Details explaining why permission from the land owner has not been obtained for the advertisement display</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
-      <c r="B64" s="2" t="n"/>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Declaration</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Signed and dated verification of the application's accuracy.</t>
+        </is>
+      </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Declaration date</t>
+          <t>Person reference</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr"/>
@@ -2567,12 +2607,12 @@
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>The date the declaration was made</t>
+          <t>Declaration must be made by an applicant or agent making the application</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -2582,19 +2622,11 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>Pre-application advice</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Details of pre-application advice previously received from the planning authority</t>
-        </is>
-      </c>
+      <c r="A65" s="2" t="n"/>
+      <c r="B65" s="2" t="n"/>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>Pre-application advice sought</t>
+          <t>Declaration confirmed</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr"/>
@@ -2602,7 +2634,7 @@
       <c r="F65" s="2" t="inlineStr"/>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Whether pre-application advice has been sought from the planning authority</t>
+          <t>Confirms the applicant or agent has reviewed and validated the information provided in the application</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -2621,7 +2653,7 @@
       <c r="B66" s="2" t="n"/>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Officer name</t>
+          <t>Declaration date</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr"/>
@@ -2629,26 +2661,34 @@
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Name of the planning officer who provided the pre-application advice</t>
+          <t>The date the declaration was made</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I66" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
-      <c r="B67" s="2" t="n"/>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Pre-application advice</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Details of pre-application advice previously received from the planning authority</t>
+        </is>
+      </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>Pre-application advice sought</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr"/>
@@ -2656,17 +2696,17 @@
       <c r="F67" s="2" t="inlineStr"/>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>A unique reference for the data item</t>
+          <t>Whether pre-application advice has been sought from the planning authority</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2715,7 @@
       <c r="B68" s="2" t="n"/>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Advice date</t>
+          <t>Officer name</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr"/>
@@ -2683,12 +2723,12 @@
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
+          <t>Name of the planning officer who provided the pre-application advice</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>datetime</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr">
@@ -2702,7 +2742,7 @@
       <c r="B69" s="2" t="n"/>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Advice summary</t>
+          <t>Reference</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr"/>
@@ -2710,7 +2750,7 @@
       <c r="F69" s="2" t="inlineStr"/>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>Summary of the pre-application advice received from the planning authority</t>
+          <t>A unique reference for the data item</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr">
@@ -2725,36 +2765,24 @@
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Proposed advert details</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Details of the proposed advertisements such as their size and how they are made</t>
-        </is>
-      </c>
+      <c r="A70" s="2" t="n"/>
+      <c r="B70" s="2" t="n"/>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Advertisements[]</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Height from ground</t>
-        </is>
-      </c>
+          <t>Advice date</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr"/>
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Height, in metres, from ground to the base of the advertisement</t>
+          <t>Date when pre-application advice was received, in YYYY-MM-DD format</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>datetime</t>
         </is>
       </c>
       <c r="I70" s="2" t="inlineStr">
@@ -2768,24 +2796,20 @@
       <c r="B71" s="2" t="n"/>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Advertisements[]</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>Height</t>
-        </is>
-      </c>
+          <t>Advice summary</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr"/>
       <c r="E71" s="2" t="inlineStr"/>
       <c r="F71" s="2" t="inlineStr"/>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Height, in metres, of dimensions of advertisement</t>
+          <t>Summary of the pre-application advice received from the planning authority</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I71" s="2" t="inlineStr">
@@ -2795,8 +2819,16 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
-      <c r="B72" s="2" t="n"/>
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Proposed advert details</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Details of the proposed advertisements such as their size and how they are made</t>
+        </is>
+      </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
           <t>Advertisements[]</t>
@@ -2804,14 +2836,14 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Width</t>
+          <t>Height from ground</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Width of dimensions of advertisement</t>
+          <t>Height, in metres, from ground to the base of the advertisement</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -2835,14 +2867,14 @@
       </c>
       <c r="D73" s="2" t="inlineStr">
         <is>
-          <t>Depth</t>
+          <t>Height</t>
         </is>
       </c>
       <c r="E73" s="2" t="inlineStr"/>
       <c r="F73" s="2" t="inlineStr"/>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Depth, in metres, of dimensions of advertisement</t>
+          <t>Height, in metres, of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -2866,14 +2898,14 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>Symbol height max</t>
+          <t>Width</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Maximum height, in metres, of any individual letters or symbols</t>
+          <t>Width of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -2897,19 +2929,19 @@
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Depth</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr"/>
       <c r="F75" s="2" t="inlineStr"/>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Colour of proposed sign</t>
+          <t>Depth, in metres, of dimensions of advertisement</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -2928,19 +2960,19 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>Materials</t>
+          <t>Symbol height max</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Materials of proposed sign</t>
+          <t>Maximum height, in metres, of any individual letters or symbols</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I76" s="2" t="inlineStr">
@@ -2959,19 +2991,19 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>Max projection</t>
+          <t>Colour</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
       <c r="F77" s="2" t="inlineStr"/>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Maximum projection, in metres, of the advertisement from the face of the building</t>
+          <t>Colour of proposed sign</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I77" s="2" t="inlineStr">
@@ -2990,19 +3022,19 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Illuminated</t>
+          <t>Materials</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Will the sign(s) be illuminated?</t>
+          <t>Materials of proposed sign</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I78" s="2" t="inlineStr">
@@ -3021,19 +3053,19 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t>Illumination method</t>
+          <t>Max projection</t>
         </is>
       </c>
       <c r="E79" s="2" t="inlineStr"/>
       <c r="F79" s="2" t="inlineStr"/>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Method of illumination for the advertisement</t>
+          <t>Maximum projection, in metres, of the advertisement from the face of the building</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I79" s="2" t="inlineStr">
@@ -3052,19 +3084,19 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>Illuminance level</t>
+          <t>Illuminated</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Level of illuminance for the advertisement</t>
+          <t>Will the sign(s) be illuminated?</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I80" s="2" t="inlineStr">
@@ -3083,14 +3115,14 @@
       </c>
       <c r="D81" s="2" t="inlineStr">
         <is>
-          <t>Illumination type</t>
+          <t>Illumination method</t>
         </is>
       </c>
       <c r="E81" s="2" t="inlineStr"/>
       <c r="F81" s="2" t="inlineStr"/>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Type of illumination (static or intermittent)</t>
+          <t>Method of illumination for the advertisement</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -3105,36 +3137,28 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Site details</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>Where the proposed development will be built.</t>
-        </is>
-      </c>
+      <c r="A82" s="2" t="n"/>
+      <c r="B82" s="2" t="n"/>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
+          <t>Advertisements[]</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Site boundary</t>
+          <t>Illuminance level</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Geometry of the site of the development, typically in GeoJSON format</t>
+          <t>Level of illuminance for the advertisement</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
         <is>
-          <t>wkt</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I82" s="2" t="inlineStr">
@@ -3148,24 +3172,24 @@
       <c r="B83" s="2" t="n"/>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>Site locations[]</t>
+          <t>Advertisements[]</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Address Text</t>
+          <t>Illumination type</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr"/>
       <c r="F83" s="2" t="inlineStr"/>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Flexible field for capturing addresses</t>
+          <t>Type of illumination (static or intermittent)</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I83" s="2" t="inlineStr">
@@ -3175,8 +3199,16 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n"/>
-      <c r="B84" s="2" t="n"/>
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Site details</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>Where the proposed development will be built.</t>
+        </is>
+      </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Site locations[]</t>
@@ -3184,24 +3216,24 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Postcode</t>
+          <t>Site boundary</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>The postal code</t>
+          <t>A polygon or multipolygon boundary</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>multipolygon</t>
         </is>
       </c>
       <c r="I84" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3215,24 +3247,28 @@
       </c>
       <c r="D85" s="2" t="inlineStr">
         <is>
-          <t>Easting</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr"/>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>Address Text</t>
+        </is>
+      </c>
       <c r="F85" s="2" t="inlineStr"/>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
+          <t>Text representation of an address or site</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3246,19 +3282,23 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Northing</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr"/>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>Postcode</t>
+        </is>
+      </c>
       <c r="F86" s="2" t="inlineStr"/>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
+          <t>Postcode for a contact address or site</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I86" s="2" t="inlineStr">
@@ -3277,19 +3317,23 @@
       </c>
       <c r="D87" s="2" t="inlineStr">
         <is>
-          <t>Latitude</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr"/>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="E87" s="2" t="inlineStr">
+        <is>
+          <t>UPRNs[]</t>
+        </is>
+      </c>
       <c r="F87" s="2" t="inlineStr"/>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Unique Property Reference Numbers (UPRNs) for existing premises within a site boundary</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I87" s="2" t="inlineStr">
@@ -3308,19 +3352,23 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Longitude</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr"/>
+          <t>Site address</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>USRNs[]</t>
+        </is>
+      </c>
       <c r="F88" s="2" t="inlineStr"/>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
+          <t>Unique Street Reference Numbers (USRNs) associated with the site</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>string</t>
         </is>
       </c>
       <c r="I88" s="2" t="inlineStr">
@@ -3339,19 +3387,19 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Easting</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="inlineStr"/>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>A text description providing details about the subject.</t>
+          <t>Easting coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I89" s="2" t="inlineStr">
@@ -3370,19 +3418,19 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>UPRNs[]</t>
+          <t>Northing</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Unique Property Reference Numbers (UPRNs) for properties within the site boundary</t>
+          <t>Northing coordinate in British National Grid (EPSG:27700)</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="I90" s="2" t="inlineStr">
@@ -3392,37 +3440,33 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>Site Visit Details</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>Information to help the planning authority arrange a site visit</t>
-        </is>
-      </c>
+      <c r="A91" s="2" t="n"/>
+      <c r="B91" s="2" t="n"/>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Site seen from public area</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr"/>
+          <t>Site locations[]</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Latitude</t>
+        </is>
+      </c>
       <c r="E91" s="2" t="inlineStr"/>
       <c r="F91" s="2" t="inlineStr"/>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
+          <t>Latitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>boolean</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I91" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -3431,34 +3475,46 @@
       <c r="B92" s="2" t="n"/>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Site visit contact type</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr"/>
+          <t>Site locations[]</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Longitude</t>
+        </is>
+      </c>
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Indicates who the authority should contact to arrange a site visit</t>
+          <t>Longitude coordinate in WGS84 (EPSG:4326)</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
         <is>
-          <t>enum</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n"/>
-      <c r="B93" s="2" t="n"/>
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>Site Visit Details</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
+          <t>Information to help the planning authority arrange a site visit</t>
+        </is>
+      </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Contact reference</t>
+          <t>Site seen from public area</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr"/>
@@ -3466,17 +3522,17 @@
       <c r="F93" s="2" t="inlineStr"/>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>The reference of the applicant or agent who should be contacted for site visits</t>
+          <t>Can site be seen from a public road, public footpath, bridleway or other public land</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>boolean</t>
         </is>
       </c>
       <c r="I93" s="2" t="inlineStr">
         <is>
-          <t>MAY</t>
+          <t>MUST</t>
         </is>
       </c>
     </row>
@@ -3485,24 +3541,20 @@
       <c r="B94" s="2" t="n"/>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>Full name</t>
-        </is>
-      </c>
+          <t>Site visit contact type</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr"/>
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>The complete name of a person</t>
+          <t>Indicates who the authority should contact to arrange a site visit</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>enum</t>
         </is>
       </c>
       <c r="I94" s="2" t="inlineStr">
@@ -3516,19 +3568,15 @@
       <c r="B95" s="2" t="n"/>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Other site visit contact</t>
-        </is>
-      </c>
-      <c r="D95" s="2" t="inlineStr">
-        <is>
-          <t>Phone number</t>
-        </is>
-      </c>
+          <t>Contact reference</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr"/>
       <c r="E95" s="2" t="inlineStr"/>
       <c r="F95" s="2" t="inlineStr"/>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>A phone number</t>
+          <t>The reference of the applicant or agent who should be contacted for site visits</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -3538,7 +3586,7 @@
       </c>
       <c r="I95" s="2" t="inlineStr">
         <is>
-          <t>MUST</t>
+          <t>MAY</t>
         </is>
       </c>
     </row>
@@ -3552,22 +3600,84 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>Full name</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr"/>
       <c r="G96" s="2" t="inlineStr">
         <is>
+          <t>The complete name of a person</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n"/>
+      <c r="B97" s="2" t="n"/>
+      <c r="C97" s="2" t="inlineStr">
+        <is>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>Phone number</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>A phone number</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
+        <is>
+          <t>MUST</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n"/>
+      <c r="B98" s="2" t="n"/>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>Other site visit contact</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
           <t>The email address that can be used for electronic correspondence with the individual</t>
         </is>
       </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
         <is>
           <t>MUST</t>
         </is>
@@ -3575,40 +3685,40 @@
     </row>
   </sheetData>
   <mergeCells count="34">
-    <mergeCell ref="A35:A42"/>
     <mergeCell ref="B31:B34"/>
-    <mergeCell ref="B35:B42"/>
-    <mergeCell ref="A53"/>
-    <mergeCell ref="B91:B96"/>
-    <mergeCell ref="B65:B69"/>
-    <mergeCell ref="B82:B90"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55"/>
     <mergeCell ref="A20:A24"/>
     <mergeCell ref="A2:A19"/>
-    <mergeCell ref="A54:A55"/>
     <mergeCell ref="B27:B30"/>
-    <mergeCell ref="A62:A64"/>
-    <mergeCell ref="B47:B52"/>
-    <mergeCell ref="A59:A61"/>
-    <mergeCell ref="B43:B46"/>
+    <mergeCell ref="B93:B98"/>
+    <mergeCell ref="B84:B92"/>
+    <mergeCell ref="A58:A60"/>
+    <mergeCell ref="A56:A57"/>
     <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B64:B66"/>
     <mergeCell ref="B20:B24"/>
-    <mergeCell ref="B56:B58"/>
-    <mergeCell ref="B59:B61"/>
+    <mergeCell ref="A64:A66"/>
+    <mergeCell ref="B72:B83"/>
     <mergeCell ref="A27:A30"/>
-    <mergeCell ref="B62:B64"/>
-    <mergeCell ref="A70:A81"/>
-    <mergeCell ref="A91:A96"/>
-    <mergeCell ref="A82:A90"/>
-    <mergeCell ref="A47:A52"/>
-    <mergeCell ref="B54:B55"/>
-    <mergeCell ref="B70:B81"/>
+    <mergeCell ref="B44:B47"/>
+    <mergeCell ref="A67:A71"/>
+    <mergeCell ref="A35:A43"/>
+    <mergeCell ref="A61:A63"/>
+    <mergeCell ref="B35:B43"/>
+    <mergeCell ref="B58:B60"/>
+    <mergeCell ref="A48:A54"/>
+    <mergeCell ref="A44:A47"/>
+    <mergeCell ref="B61:B63"/>
+    <mergeCell ref="B67:B71"/>
     <mergeCell ref="A31:A34"/>
-    <mergeCell ref="A43:A46"/>
-    <mergeCell ref="B53"/>
-    <mergeCell ref="A65:A69"/>
+    <mergeCell ref="A55"/>
+    <mergeCell ref="B56:B57"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="B2:B19"/>
-    <mergeCell ref="A56:A58"/>
+    <mergeCell ref="A72:A83"/>
+    <mergeCell ref="A93:A98"/>
+    <mergeCell ref="A84:A92"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>